<commit_message>
Update patient catalog and enhance documentation for operational governance
- Updated `ddc-master_patient_catalog.parquet` to reflect the latest schema changes.
- Revised `README.md` to include references to the new `docs/operational-runbook.md`, detailing Level A production roles and processes.
- Enhanced `docs/demographics-pilot-plan.md` to clarify steward assignments and governance content progress.
- Updated `docs/documentation-map.md` to include the operational runbook for better navigation.
- Modified `scripts/generate_steward_workbook.py` and `scripts/seed_demographics_pilot.py` to reflect updated steward assignments and contact information.
</commit_message>
<xml_diff>
--- a/workbooks/chi-steward-workbook.xlsx
+++ b/workbooks/chi-steward-workbook.xlsx
@@ -16580,7 +16580,7 @@
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="17" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
     <col width="38" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
@@ -16643,7 +16643,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>SHIE Data Governance</t>
+          <t>Ajay Prashar</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -16681,7 +16681,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>SHIE Data Governance</t>
+          <t>Ajay Prashar</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -16719,7 +16719,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>SHIE Data Governance</t>
+          <t>Ajay Prashar</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -16757,7 +16757,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>SHIE Data Governance</t>
+          <t>Ajay Prashar</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -16795,7 +16795,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>SHIE Data Governance</t>
+          <t>Ajay Prashar</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -18942,8 +18942,8 @@
     <col width="21" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="17" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
-    <col width="17" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
     <col width="17" customWidth="1" min="12" max="12"/>
     <col width="16" customWidth="1" min="13" max="13"/>
     <col width="20" customWidth="1" min="14" max="14"/>
@@ -19396,10 +19396,14 @@
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr">
         <is>
-          <t>SHIE Data Governance</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr"/>
+          <t>Ajay Prashar</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Ajay.Prashar@acgov.org</t>
+        </is>
+      </c>
       <c r="L9" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -19459,10 +19463,14 @@
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr">
         <is>
-          <t>SHIE Data Governance</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr"/>
+          <t>Ajay Prashar</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Ajay.Prashar@acgov.org</t>
+        </is>
+      </c>
       <c r="L10" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -19565,10 +19573,14 @@
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr">
         <is>
-          <t>SHIE Data Governance</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr"/>
+          <t>Ajay Prashar</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Ajay.Prashar@acgov.org</t>
+        </is>
+      </c>
       <c r="L12" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -19628,10 +19640,14 @@
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr">
         <is>
-          <t>SHIE Data Governance</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr"/>
+          <t>Ajay Prashar</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Ajay.Prashar@acgov.org</t>
+        </is>
+      </c>
       <c r="L13" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -19691,10 +19707,14 @@
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr">
         <is>
-          <t>SHIE Data Governance</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr"/>
+          <t>Ajay Prashar</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Ajay.Prashar@acgov.org</t>
+        </is>
+      </c>
       <c r="L14" t="inlineStr">
         <is>
           <t>Approved</t>

</xml_diff>

<commit_message>
Add value set and crosswalk layer; PBIP standards tables and report formatting
</commit_message>
<xml_diff>
--- a/workbooks/chi-steward-workbook.xlsx
+++ b/workbooks/chi-steward-workbook.xlsx
@@ -18,9 +18,12 @@
     <sheet name="CCDA_Mappings" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="FHIR_Inventory" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="Business_Rules" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Source_Registry" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Steward_Queue" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Concept_Explorer" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Value_Set_Bindings" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Value_Set_Members" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Source_Value_Crosswalk" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Source_Registry" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Steward_Queue" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Concept_Explorer" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -178,8 +181,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="chi_table_index" displayName="chi_table_index" ref="A1:D13" headerRowCount="1">
-  <autoFilter ref="A1:D13"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="chi_table_index" displayName="chi_table_index" ref="A1:D16" headerRowCount="1">
+  <autoFilter ref="A1:D16"/>
   <tableColumns count="4">
     <tableColumn id="1" name="excel_table_name"/>
     <tableColumn id="2" name="sheet_tab"/>
@@ -191,7 +194,68 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="chi_source_registry" displayName="chi_source_registry" ref="A1:E2" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="chi_value_set_binding" displayName="chi_value_set_binding" ref="A1:K6" headerRowCount="1">
+  <autoFilter ref="A1:K6"/>
+  <tableColumns count="11">
+    <tableColumn id="1" name="semantic_id"/>
+    <tableColumn id="2" name="binding_role"/>
+    <tableColumn id="3" name="value_set_name"/>
+    <tableColumn id="4" name="value_set_url"/>
+    <tableColumn id="5" name="code_system_oid"/>
+    <tableColumn id="6" name="code_system_name"/>
+    <tableColumn id="7" name="binding_strength"/>
+    <tableColumn id="8" name="fhir_element"/>
+    <tableColumn id="9" name="authority_reference"/>
+    <tableColumn id="10" name="approval_status"/>
+    <tableColumn id="11" name="notes"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="chi_value_set_member" displayName="chi_value_set_member" ref="A1:J22" headerRowCount="1">
+  <autoFilter ref="A1:J22"/>
+  <tableColumns count="10">
+    <tableColumn id="1" name="semantic_id"/>
+    <tableColumn id="2" name="code_system_oid"/>
+    <tableColumn id="3" name="code"/>
+    <tableColumn id="4" name="display"/>
+    <tableColumn id="5" name="member_type"/>
+    <tableColumn id="6" name="binding_role"/>
+    <tableColumn id="7" name="binding_strength"/>
+    <tableColumn id="8" name="active"/>
+    <tableColumn id="9" name="sort_order"/>
+    <tableColumn id="10" name="notes"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="chi_source_value_crosswalk" displayName="chi_source_value_crosswalk" ref="A1:M5" headerRowCount="1">
+  <autoFilter ref="A1:M5"/>
+  <tableColumns count="13">
+    <tableColumn id="1" name="source_id"/>
+    <tableColumn id="2" name="source_field"/>
+    <tableColumn id="3" name="source_code"/>
+    <tableColumn id="4" name="source_display"/>
+    <tableColumn id="5" name="semantic_id"/>
+    <tableColumn id="6" name="target_code_system_oid"/>
+    <tableColumn id="7" name="target_code"/>
+    <tableColumn id="8" name="target_display"/>
+    <tableColumn id="9" name="mapping_type"/>
+    <tableColumn id="10" name="approval_status"/>
+    <tableColumn id="11" name="effective_from"/>
+    <tableColumn id="12" name="effective_to"/>
+    <tableColumn id="13" name="notes"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="chi_source_registry" displayName="chi_source_registry" ref="A1:E2" headerRowCount="1">
   <autoFilter ref="A1:E2"/>
   <tableColumns count="5">
     <tableColumn id="1" name="source_id"/>
@@ -204,8 +268,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="chi_steward_queue" displayName="chi_steward_queue" ref="A1:H47" headerRowCount="1">
+<file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="chi_steward_queue" displayName="chi_steward_queue" ref="A1:H47" headerRowCount="1">
   <autoFilter ref="A1:H47"/>
   <tableColumns count="8">
     <tableColumn id="1" name="semantic_id"/>
@@ -16509,6 +16573,1878 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:K6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="37" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="38" customWidth="1" min="8" max="8"/>
+    <col width="38" customWidth="1" min="9" max="9"/>
+    <col width="17" customWidth="1" min="10" max="10"/>
+    <col width="38" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>semantic_id</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>binding_role</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>value_set_name</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>value_set_url</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>code_system_oid</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>code_system_name</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>binding_strength</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>fhir_element</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>authority_reference</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>approval_status</t>
+        </is>
+      </c>
+      <c r="K1" s="4" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Patient.race</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>HL7 Race</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>http://terminology.hl7.org/ValueSet/v3-Race</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>urn:oid:2.16.840.1.113883.6.238</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>CDCREC</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>required</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Patient.extension(us-core-race).ombCategory</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>docs/shie-standards-reference.md#cdcrec-race-codes-omb-rollup-examples</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>US Core us-core-race: ombCategory required; detailed optional.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Patient.ethnicity</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>HL7 Ethnicity</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>http://terminology.hl7.org/ValueSet/v3-Ethnicity</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>urn:oid:2.16.840.1.113883.6.238</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>CDCREC</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>required</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Patient.extension(us-core-ethnicity).ombCategory</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>docs/shie-standards-reference.md#cdcrec-ethnicity-codes-examples</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>US Core us-core-ethnicity extension.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Patient.language</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>FHIR Languages (BCP 47)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>http://hl7.org/fhir/ValueSet/languages</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>urn:ietf:bcp:47</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>BCP 47</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>required</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Patient.communication.language</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>docs/shie-standards-reference.md</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Primary FHIR binding; ISO 639 for stewardship crosswalk only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Patient.gender_id</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>US Core Gender Identity Observation</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>http://hl7.org/fhir/us/core/StructureDefinition/us-core-observation-social-history</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>urn:oid:2.16.840.1.113883.6.1</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>LOINC</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>required</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Observation.code (LOINC 76691-5)</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>docs/shie-standards-reference.md</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Answer values often SNOMED-coded; expand members from US Core / partner intake.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Patient.birth_sex</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>US Core Birth Sex</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>http://hl7.org/fhir/us/core/StructureDefinition/us-core-birthsex</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>http://hl7.org/fhir/us/core/CodeSystem/birthsex</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>US Core birth sex</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>required</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Patient.extension(us-core-birthsex)</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>docs/shie-standards-reference.md</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Administrative sex — not CDCREC; distinct from gender identity.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="38" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>semantic_id</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>code_system_oid</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>display</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>member_type</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>binding_role</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>binding_strength</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>sort_order</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Patient.race</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>urn:oid:2.16.840.1.113883.6.238</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1002-5</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>American Indian or Alaska Native</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>omb_rollup</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>required</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>HL7 Race Value Set / CDC PHIN reporting rollup</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Patient.race</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>urn:oid:2.16.840.1.113883.6.238</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2028-9</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Asian</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>omb_rollup</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>required</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>HL7 Race Value Set / CDC PHIN reporting rollup</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Patient.race</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>urn:oid:2.16.840.1.113883.6.238</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2054-5</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Black or African American</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>omb_rollup</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>required</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>HL7 Race Value Set / CDC PHIN reporting rollup</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Patient.race</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>urn:oid:2.16.840.1.113883.6.238</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2076-8</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Native Hawaiian or Other Pacific Islander</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>omb_rollup</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>required</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>HL7 Race Value Set / CDC PHIN reporting rollup</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Patient.race</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>urn:oid:2.16.840.1.113883.6.238</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2106-3</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>White</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>omb_rollup</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>required</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>HL7 Race Value Set / CDC PHIN reporting rollup</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Patient.race</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>urn:oid:2.16.840.1.113883.6.238</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2131-1</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Other Race</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>omb_rollup</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>required</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>HL7 Race Value Set / CDC PHIN reporting rollup</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Patient.race</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>urn:oid:2.16.840.1.113883.5.1008</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>UNK</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>nullflavor</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>nullflavor</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>example</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Do not collapse with valid race codes in reporting</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Patient.race</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>urn:oid:2.16.840.1.113883.5.1008</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>ASKU</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Asked but not known</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>nullflavor</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>nullflavor</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>example</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Do not collapse with valid race codes in reporting</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Patient.race</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>urn:oid:2.16.840.1.113883.5.1008</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>NASK</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Not asked</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>nullflavor</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>nullflavor</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>example</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Do not collapse with valid race codes in reporting</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Patient.ethnicity</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>urn:oid:2.16.840.1.113883.6.238</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2135-2</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Hispanic or Latino</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>omb_rollup</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>required</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Patient.ethnicity</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>urn:oid:2.16.840.1.113883.6.238</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>2186-5</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Not Hispanic or Latino</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>omb_rollup</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>required</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Patient.ethnicity</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>urn:oid:2.16.840.1.113883.5.1008</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>UNK</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>nullflavor</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>nullflavor</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>example</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Distinct from patient-refused / declined in survivorship</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Patient.language</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>urn:ietf:bcp:47</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>language_tag</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>example</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Pilot examples; full list from IANA/BCP 47 — not duplicated locally</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Patient.language</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>urn:ietf:bcp:47</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Spanish</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>language_tag</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>example</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Pilot examples; full list from IANA/BCP 47 — not duplicated locally</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Patient.language</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>urn:ietf:bcp:47</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>zh</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Chinese</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>language_tag</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>example</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Pilot examples; full list from IANA/BCP 47 — not duplicated locally</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Patient.language</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>urn:ietf:bcp:47</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>vi</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Vietnamese</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>language_tag</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>example</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Pilot examples; full list from IANA/BCP 47 — not duplicated locally</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Patient.language</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>urn:ietf:bcp:47</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Arabic</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>language_tag</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>example</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Pilot examples; full list from IANA/BCP 47 — not duplicated locally</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Patient.language</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>urn:ietf:bcp:47</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>und</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Undetermined</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>example</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Excluded from county aggregates per survivorship</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Patient.birth_sex</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>http://hl7.org/fhir/us/core/CodeSystem/birthsex</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>administrative</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>required</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Not interchangeable with Patient.gender_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Patient.birth_sex</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>http://hl7.org/fhir/us/core/CodeSystem/birthsex</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>administrative</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>required</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Not interchangeable with Patient.gender_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Patient.birth_sex</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>http://hl7.org/fhir/us/core/CodeSystem/birthsex</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>UNK</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>administrative</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>required</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Not interchangeable with Patient.gender_id</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="38" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="27" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="17" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="38" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>source_id</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>source_field</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>source_code</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>source_display</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>semantic_id</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>target_code_system_oid</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>target_code</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>target_display</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>mapping_type</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>approval_status</t>
+        </is>
+      </c>
+      <c r="K1" s="4" t="inlineStr">
+        <is>
+          <t>effective_from</t>
+        </is>
+      </c>
+      <c r="L1" s="4" t="inlineStr">
+        <is>
+          <t>effective_to</t>
+        </is>
+      </c>
+      <c r="M1" s="4" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>cmt</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>PID-10</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>EXAMPLE_B</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>CMT race code (replace with validated list)</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Patient.race</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>urn:oid:2.16.840.1.113883.6.238</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2054-5</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Black or African American</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>rollup</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>POC placeholder — populate from CMT race code inventory / county Table 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>cmt</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>PID-22</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>EXAMPLE_H</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>CMT ethnicity code (replace with validated list)</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Patient.ethnicity</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>urn:oid:2.16.840.1.113883.6.238</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2135-2</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Hispanic or Latino</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>rollup</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>POC placeholder — populate from CMT ethnicity code inventory</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>cmt</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>PID-15</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Patient.language</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>urn:ietf:bcp:47</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Example exact map when CMT sends BCP 47 or ISO-aligned language code</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>cmt</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>PID-8</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Patient.birth_sex</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>http://hl7.org/fhir/us/core/CodeSystem/birthsex</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Administrative sex / SexID — not gender identity</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -16569,7 +18505,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -17402,13 +19338,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -17599,21 +19535,54 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
+          <t>Governed code (first member)</t>
+        </is>
+      </c>
+      <c r="B18" s="2">
+        <f>IF($B$3="","",IFERROR(INDEX(chi_value_set_member[code],MATCH($B$3,chi_value_set_member[semantic_id],0)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Governed code display (first member)</t>
+        </is>
+      </c>
+      <c r="B19" s="2">
+        <f>IF($B$3="","",IFERROR(INDEX(chi_value_set_member[display],MATCH($B$3,chi_value_set_member[semantic_id],0)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Source crosswalk code (first match)</t>
+        </is>
+      </c>
+      <c r="B20" s="2">
+        <f>IF($B$3="","",IFERROR(INDEX(chi_source_value_crosswalk[source_code],MATCH($B$3,chi_source_value_crosswalk[semantic_id],0)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
           <t>Primary source (first link)</t>
         </is>
       </c>
-      <c r="B18" s="2">
+      <c r="B21" s="2">
         <f>IF($B$3="","",IFERROR(INDEX(chi_source_availability[source_id],MATCH($B$3,chi_source_availability[semantic_id],0)),""))</f>
         <v/>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
+    <row r="22">
+      <c r="A22" t="inlineStr">
         <is>
           <t>Source availability</t>
         </is>
       </c>
-      <c r="B19" s="2">
+      <c r="B22" s="2">
         <f>IF($B$3="","",IFERROR(INDEX(chi_source_availability[availability],MATCH($B$3,chi_source_availability[semantic_id],0)),""))</f>
         <v/>
       </c>
@@ -17629,13 +19598,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="38" customWidth="1" min="7" max="7"/>
@@ -17903,35 +19872,146 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>catalog_value_set_binding</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>chi_catalog</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>semantic_id</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>chi_value_set_binding</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>semantic_id</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>1:N</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Which terminology / value set applies to the concept.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>catalog_value_set_member</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>chi_catalog</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>semantic_id</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>chi_value_set_member</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>semantic_id</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>1:N</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Governed codes for the concept (CHI subset).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>catalog_source_crosswalk</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>chi_catalog</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>semantic_id</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>chi_source_value_crosswalk</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>semantic_id</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>1:N</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Source-local values mapped to governed standard codes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>catalog_steward_queue</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>chi_catalog</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>semantic_id</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>chi_steward_queue</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>semantic_id</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>1:1</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>Optional steward workflow overlay keyed by semantic_id.</t>
         </is>
@@ -17948,11 +20028,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
     <col width="38" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
   </cols>
@@ -18202,42 +20282,108 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>chi_lookup_lists</t>
+          <t>chi_value_set_binding</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Lookup_Lists</t>
+          <t>Value_Set_Bindings</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>(reference lists)</t>
+          <t>ddc-value_set_binding.parquet</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Reference</t>
+          <t>Terminology</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>chi_value_set_member</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Value_Set_Members</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>ddc-value_set_member.parquet</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Terminology</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>chi_source_value_crosswalk</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Source_Value_Crosswalk</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>ddc-source_value_crosswalk.parquet</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Crosswalk</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>chi_lookup_lists</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Lookup_Lists</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>(reference lists)</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
           <t>chi_table_index</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>Table_Index</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>(navigation map; not imported)</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>Reference</t>
         </is>

</xml_diff>